<commit_message>
Fix: Excel con formato original exacto - colores, bordes, márgenes copiados del original
</commit_message>
<xml_diff>
--- a/template_cargue.xlsx
+++ b/template_cargue.xlsx
@@ -16,8 +16,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,23 +31,50 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <sz val="11"/>
+      <sz val="20"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <sz val="10"/>
+      <sz val="14"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.7999816888943144"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -50,16 +82,176 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,91 +617,138 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:M5"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="1.66" customWidth="1" min="1" max="1"/>
+    <col width="1.6640625" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="11.44" customWidth="1" min="3" max="3"/>
-    <col width="9.109999999999999" customWidth="1" min="4" max="4"/>
-    <col width="13.11" customWidth="1" min="5" max="5"/>
-    <col width="16.66" customWidth="1" min="6" max="6"/>
-    <col width="12.66" customWidth="1" min="7" max="7"/>
-    <col width="24.33" customWidth="1" min="8" max="8"/>
-    <col width="11.55" customWidth="1" min="9" max="9"/>
-    <col width="16.66" customWidth="1" min="10" max="10"/>
-    <col width="15.33" customWidth="1" min="11" max="11"/>
+    <col width="11.44140625" customWidth="1" min="3" max="3"/>
+    <col width="9.109375" customWidth="1" min="4" max="4"/>
+    <col width="13.109375" customWidth="1" min="5" max="5"/>
+    <col width="16.6640625" customWidth="1" min="6" max="6"/>
+    <col width="12.6640625" customWidth="1" min="7" max="7"/>
+    <col width="24.33203125" customWidth="1" min="8" max="8"/>
+    <col width="11.5546875" customWidth="1" min="9" max="9"/>
+    <col width="16.6640625" customWidth="1" min="10" max="10"/>
+    <col width="15.33203125" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="14.44" customWidth="1" min="13" max="13"/>
-    <col width="23.44" customWidth="1" min="14" max="14"/>
+    <col width="14.44140625" customWidth="1" min="13" max="13"/>
+    <col width="23.44140625" customWidth="1" min="14" max="14"/>
+    <col width="9.44140625" customWidth="1" min="15" max="15"/>
+    <col width="33.5546875" customWidth="1" min="16" max="16"/>
+    <col width="13.88671875" customWidth="1" min="17" max="17"/>
+    <col width="20.6640625" customWidth="1" min="18" max="18"/>
+    <col width="15.5546875" customWidth="1" min="19" max="19"/>
+    <col width="13.88671875" customWidth="1" min="20" max="20"/>
+    <col width="13.88671875" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="E3" s="1" t="inlineStr">
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3" ht="22.2" customHeight="1">
+      <c r="C3" s="1" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">                             REPORTE DIARIO DE CARGUE  SAVICOL</t>
         </is>
       </c>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="5" t="n"/>
+      <c r="M3" s="2" t="n"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr">
+    <row r="4" ht="11.4" customHeight="1">
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="1" t="n"/>
+      <c r="L4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="47.4" customHeight="1">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">FECHA </t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Nº VIAJES</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">GRANJA </t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>CUADRILLA</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">CANTIDAD DE PERSONAS </t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="13" t="inlineStr">
         <is>
           <t>NOMBRE CONDUCTOR</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="15" t="inlineStr">
         <is>
           <t>HORA INICIO</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">HORA SALIDA </t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L5" s="17" t="inlineStr">
         <is>
           <t>CANTIDAD</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M5" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL POLLOS DIA </t>
         </is>
       </c>
+      <c r="P5" s="19" t="n"/>
+      <c r="Q5" s="19" t="n"/>
+      <c r="R5" s="19" t="n"/>
+      <c r="S5" s="19" t="n"/>
+      <c r="T5" s="19" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="C6" s="20" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="n"/>
+      <c r="G6" s="22" t="n"/>
+      <c r="H6" s="22" t="n"/>
+      <c r="I6" s="22" t="n"/>
+      <c r="J6" s="22" t="n"/>
+      <c r="K6" s="23" t="n"/>
+      <c r="L6" s="24" t="n"/>
+      <c r="M6" s="25" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>